<commit_message>
feat: update project SGI documentation, add visual assets, and implement remark plugins for image handling and language tabs
</commit_message>
<xml_diff>
--- a/public/documents/E6/Gestion_Projet_App_SGI.xlsx
+++ b/public/documents/E6/Gestion_Projet_App_SGI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wblondel/my-portfolio/public/documents/E6/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wblondel/kDrive/BTS SIO/Application SGI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320A20B2-8EDA-FF44-B50B-B6A95532F4AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41287126-2301-3446-9F59-EFD209BF2291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20580" yWindow="780" windowWidth="20560" windowHeight="25800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Stories" sheetId="1" r:id="rId1"/>
@@ -170,9 +170,6 @@
     <t>US-12</t>
   </si>
   <si>
-    <t>Securite</t>
-  </si>
-  <si>
     <t>- OrderPolicy: view (propres + BypassOwnership), update (demandeur si Sent + propre, admin toujours)
 - create, delete, restore, forceDelete
 - Demandeur: Create:Order ajoute au role</t>
@@ -276,9 +273,6 @@
     <t>US-24</t>
   </si>
   <si>
-    <t>Qualite</t>
-  </si>
-  <si>
     <t>- Tests unitaires : OrderStatusTest (7), OrderAgeCalculatorTest (9)
 - Tests feature : OrderPolicyTest (28), CreateOrderTest (7), ListOrdersTest (5)
 - Tests notifications : OrderNotificationTest (6)
@@ -804,6 +798,9 @@
     <t>Tests feature OrderPolicyTest</t>
   </si>
   <si>
+    <t>28 tests : CRUD admin/demandeur, cancel, processOrder, markOrdered, markReceived, closeOrder.</t>
+  </si>
+  <si>
     <t>T-055</t>
   </si>
   <si>
@@ -816,12 +813,18 @@
     <t>Tests feature ListOrdersTest</t>
   </si>
   <si>
+    <t>5 tests : page load, admin voit tout, demandeur voit propres, filtre statut.</t>
+  </si>
+  <si>
     <t>T-057</t>
   </si>
   <si>
     <t>Tests OrderNotificationTest</t>
   </si>
   <si>
+    <t>6 tests : contenu email, canaux, toArray pour OrderCreated et OrderStatusChanged.</t>
+  </si>
+  <si>
     <t>Total tickets</t>
   </si>
   <si>
@@ -904,6 +907,15 @@
   </si>
   <si>
     <t>Ajouter columnSpanFull sur les 3 sections pour empêcher le layout 2 colonnes.</t>
+  </si>
+  <si>
+    <t>7 tests : toutes les transitions valides/invalides, états terminaux, non-terminaux.</t>
+  </si>
+  <si>
+    <t>9 tests : jours ouvrés, week-ends exclus, vacances exclues, cas limites.</t>
+  </si>
+  <si>
+    <t>7 tests : création avec lignes, auto-fill user_id, statut Sent, notification admin, validations.</t>
   </si>
   <si>
     <t xml:space="preserve">  Modèles Eloquent avec relations (Order, OrderLine, Service, Supplier, Budget, Category)</t>
@@ -1251,22 +1263,10 @@
     <t>VELOCITÉ &amp; CHARGE PAR DÉVELOPPEUR</t>
   </si>
   <si>
-    <t>Tests : toutes les transitions valides/invalides, états terminaux, non-terminaux.</t>
-  </si>
-  <si>
-    <t>Tests : jours ouvrés, week-ends exclus, vacances exclues, cas limites.</t>
-  </si>
-  <si>
-    <t>Tests : CRUD admin/demandeur, cancel, processOrder, markOrdered, markReceived, closeOrder.</t>
-  </si>
-  <si>
-    <t>Tests : création avec lignes, auto-fill user_id, statut Sent, notification admin, validations.</t>
-  </si>
-  <si>
-    <t>Tests : page load, admin voit tout, demandeur voit propres, filtre statut.</t>
-  </si>
-  <si>
-    <t>Tests : contenu email, canaux, toArray pour OrderCreated et OrderStatusChanged.</t>
+    <t>Qualité</t>
+  </si>
+  <si>
+    <t>Sécurité</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1485,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1624,9 +1624,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1938,8 +1935,7 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="60" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="3" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
@@ -1967,10 +1963,10 @@
         <v>3</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>4</v>
@@ -1981,16 +1977,16 @@
     </row>
     <row r="4" spans="1:7" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>8</v>
@@ -1999,7 +1995,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="56" x14ac:dyDescent="0.2">
@@ -2010,16 +2006,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G5" s="26" t="s">
         <v>9</v>
@@ -2033,16 +2029,16 @@
         <v>7</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>9</v>
@@ -2056,10 +2052,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>288</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>370</v>
+        <v>292</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>374</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>8</v>
@@ -2079,10 +2075,10 @@
         <v>7</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>8</v>
@@ -2102,7 +2098,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>14</v>
@@ -2125,7 +2121,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>17</v>
@@ -2148,7 +2144,7 @@
         <v>20</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>21</v>
@@ -2157,7 +2153,7 @@
         <v>8</v>
       </c>
       <c r="F11" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>18</v>
@@ -2171,7 +2167,7 @@
         <v>20</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>23</v>
@@ -2180,7 +2176,7 @@
         <v>8</v>
       </c>
       <c r="F12" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>18</v>
@@ -2194,16 +2190,16 @@
         <v>20</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>18</v>
@@ -2226,7 +2222,7 @@
         <v>8</v>
       </c>
       <c r="F14" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>18</v>
@@ -2249,7 +2245,7 @@
         <v>8</v>
       </c>
       <c r="F15" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>18</v>
@@ -2260,19 +2256,19 @@
         <v>31</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>302</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F16" s="5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>18</v>
@@ -2280,62 +2276,62 @@
     </row>
     <row r="17" spans="1:7" ht="70" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="21" t="s">
+        <v>307</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>303</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F17" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>8</v>
@@ -2344,21 +2340,21 @@
         <v>2</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>8</v>
@@ -2367,200 +2363,200 @@
         <v>2</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="70" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="21" t="s">
+        <v>310</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>306</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>44</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="56" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="21" t="s">
+        <v>311</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>376</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="21" t="s">
-        <v>307</v>
-      </c>
-      <c r="D22" s="25" t="s">
-        <v>372</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>47</v>
-      </c>
       <c r="F22" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="56" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="21" t="s">
+        <v>312</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="21" t="s">
-        <v>308</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>50</v>
-      </c>
       <c r="E23" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F23" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>52</v>
-      </c>
       <c r="C24" s="21" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F24" s="5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="D25" s="25" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F25" s="5">
         <v>3</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="42" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D26" s="25" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F26" s="5">
         <v>3</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="C27" s="21" t="s">
+        <v>315</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>311</v>
-      </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="9" t="s">
         <v>60</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>61</v>
       </c>
       <c r="F27" s="5">
         <v>3</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="70" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>316</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>312</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>64</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F28" s="5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="E30" s="10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F30" s="11">
-        <f>SUM(F5:F28)</f>
-        <v>91</v>
+        <f>SUM(F4:F28)</f>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2586,7 +2582,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -2599,7 +2595,7 @@
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="41" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B3" s="37"/>
       <c r="C3" s="37"/>
@@ -2609,10 +2605,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="30" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C4" s="39"/>
       <c r="D4" s="39"/>
@@ -2621,10 +2617,10 @@
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C5" s="39"/>
       <c r="D5" s="39"/>
@@ -2633,10 +2629,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="C6" s="34"/>
       <c r="D6" s="34"/>
@@ -2658,7 +2654,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B8" s="43"/>
       <c r="C8" s="43"/>
@@ -2668,7 +2664,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="47" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B9" s="48"/>
       <c r="C9" s="48"/>
@@ -2678,7 +2674,7 @@
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="35" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B10" s="34"/>
       <c r="C10" s="34"/>
@@ -2688,7 +2684,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="35" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B11" s="34"/>
       <c r="C11" s="34"/>
@@ -2698,7 +2694,7 @@
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="47" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B12" s="48"/>
       <c r="C12" s="48"/>
@@ -2708,7 +2704,7 @@
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="44" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B14" s="45"/>
       <c r="C14" s="45"/>
@@ -2718,10 +2714,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="30" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="C15" s="39"/>
       <c r="D15" s="39"/>
@@ -2730,10 +2726,10 @@
     </row>
     <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C16" s="39"/>
       <c r="D16" s="39"/>
@@ -2742,10 +2738,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C17" s="34"/>
       <c r="D17" s="34"/>
@@ -2758,7 +2754,7 @@
       </c>
       <c r="B18" s="33" cm="1">
         <f t="array" ref="B18">SUMPRODUCT(('User Stories'!G4:G28="Sprint 1")*('User Stories'!F4:F28))</f>
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C18" s="34"/>
       <c r="D18" s="34"/>
@@ -2767,7 +2763,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B19" s="43"/>
       <c r="C19" s="43"/>
@@ -2777,7 +2773,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B20" s="34"/>
       <c r="C20" s="34"/>
@@ -2787,7 +2783,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="35" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B21" s="34"/>
       <c r="C21" s="34"/>
@@ -2797,7 +2793,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="33" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B22" s="34"/>
       <c r="C22" s="34"/>
@@ -2807,7 +2803,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B23" s="34"/>
       <c r="C23" s="34"/>
@@ -2817,7 +2813,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="35" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
@@ -2827,7 +2823,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="35" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B25" s="34"/>
       <c r="C25" s="34"/>
@@ -2837,7 +2833,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B26" s="34"/>
       <c r="C26" s="34"/>
@@ -2847,7 +2843,7 @@
     </row>
     <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="36" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B28" s="37"/>
       <c r="C28" s="37"/>
@@ -2857,10 +2853,10 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="30" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C29" s="34"/>
       <c r="D29" s="34"/>
@@ -2869,10 +2865,10 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B30" s="35" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C30" s="34"/>
       <c r="D30" s="34"/>
@@ -2881,10 +2877,10 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C31" s="34"/>
       <c r="D31" s="34"/>
@@ -2897,7 +2893,7 @@
       </c>
       <c r="B32" s="33" cm="1">
         <f t="array" ref="B32">SUMPRODUCT(('User Stories'!G4:G28="Sprint 2")*('User Stories'!F4:F28))</f>
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C32" s="34"/>
       <c r="D32" s="34"/>
@@ -2906,7 +2902,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B33" s="43"/>
       <c r="C33" s="43"/>
@@ -2916,7 +2912,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="33" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B34" s="34"/>
       <c r="C34" s="34"/>
@@ -2926,7 +2922,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B35" s="34"/>
       <c r="C35" s="34"/>
@@ -2936,7 +2932,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B36" s="34"/>
       <c r="C36" s="34"/>
@@ -2946,7 +2942,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="33" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B37" s="34"/>
       <c r="C37" s="34"/>
@@ -2956,7 +2952,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="35" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B38" s="34"/>
       <c r="C38" s="34"/>
@@ -2966,7 +2962,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="35" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B39" s="34"/>
       <c r="C39" s="34"/>
@@ -2976,7 +2972,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="33" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B40" s="34"/>
       <c r="C40" s="34"/>
@@ -2986,7 +2982,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="33" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B41" s="34"/>
       <c r="C41" s="34"/>
@@ -2996,7 +2992,7 @@
     </row>
     <row r="43" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="41" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="B43" s="37"/>
       <c r="C43" s="37"/>
@@ -3006,10 +3002,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="30" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B44" s="35" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="C44" s="34"/>
       <c r="D44" s="34"/>
@@ -3018,10 +3014,10 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B45" s="35" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C45" s="34"/>
       <c r="D45" s="34"/>
@@ -3030,10 +3026,10 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C46" s="34"/>
       <c r="D46" s="34"/>
@@ -3046,7 +3042,7 @@
       </c>
       <c r="B47" s="33" cm="1">
         <f t="array" ref="B47">SUMPRODUCT(('User Stories'!G4:G28="Sprint 3")*('User Stories'!F4:F28))</f>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C47" s="34"/>
       <c r="D47" s="34"/>
@@ -3055,7 +3051,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B48" s="43"/>
       <c r="C48" s="43"/>
@@ -3065,7 +3061,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="35" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B49" s="34"/>
       <c r="C49" s="34"/>
@@ -3075,7 +3071,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="33" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B50" s="34"/>
       <c r="C50" s="34"/>
@@ -3085,7 +3081,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="35" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B51" s="34"/>
       <c r="C51" s="34"/>
@@ -3095,7 +3091,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="33" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B52" s="34"/>
       <c r="C52" s="34"/>
@@ -3105,7 +3101,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="35" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B53" s="34"/>
       <c r="C53" s="34"/>
@@ -3115,7 +3111,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="35" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B54" s="34"/>
       <c r="C54" s="34"/>
@@ -3125,7 +3121,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="35" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B55" s="34"/>
       <c r="C55" s="34"/>
@@ -3135,7 +3131,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="35" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B56" s="34"/>
       <c r="C56" s="34"/>
@@ -3145,7 +3141,7 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="35" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B57" s="34"/>
       <c r="C57" s="34"/>
@@ -3155,7 +3151,7 @@
     </row>
     <row r="59" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="36" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B59" s="37"/>
       <c r="C59" s="37"/>
@@ -3165,10 +3161,10 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="30" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B60" s="35" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="C60" s="34"/>
       <c r="D60" s="34"/>
@@ -3177,10 +3173,10 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B61" s="35" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C61" s="34"/>
       <c r="D61" s="34"/>
@@ -3189,10 +3185,10 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B62" s="33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C62" s="34"/>
       <c r="D62" s="34"/>
@@ -3205,7 +3201,7 @@
       </c>
       <c r="B63" s="33" cm="1">
         <f t="array" ref="B63">SUMPRODUCT(('User Stories'!G4:G28="Sprint 4")*('User Stories'!F4:F28))</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C63" s="34"/>
       <c r="D63" s="34"/>
@@ -3214,7 +3210,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="42" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B64" s="43"/>
       <c r="C64" s="43"/>
@@ -3224,7 +3220,7 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="35" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B65" s="34"/>
       <c r="C65" s="34"/>
@@ -3234,7 +3230,7 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="35" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="B66" s="34"/>
       <c r="C66" s="34"/>
@@ -3244,7 +3240,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="33" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B67" s="34"/>
       <c r="C67" s="34"/>
@@ -3254,7 +3250,7 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="33" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B68" s="34"/>
       <c r="C68" s="34"/>
@@ -3264,7 +3260,7 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="33" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B69" s="34"/>
       <c r="C69" s="34"/>
@@ -3274,7 +3270,7 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="33" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B70" s="34"/>
       <c r="C70" s="34"/>
@@ -3284,7 +3280,7 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="33" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B71" s="34"/>
       <c r="C71" s="34"/>
@@ -3294,7 +3290,7 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="33" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B72" s="34"/>
       <c r="C72" s="34"/>
@@ -3391,8 +3387,8 @@
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="43" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="65" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="45" customWidth="1"/>
+    <col min="5" max="5" width="65" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="9" width="10" customWidth="1"/>
@@ -3400,7 +3396,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="49" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -3413,7 +3409,7 @@
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>5</v>
@@ -3422,201 +3418,201 @@
         <v>3</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B4" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G4" s="5">
         <v>3</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G5" s="5">
         <v>3</v>
       </c>
       <c r="H5" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G6" s="5">
         <v>2</v>
       </c>
       <c r="H6" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B7" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G7" s="5">
         <v>2</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A8" s="23" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G8" s="5">
         <v>3</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A9" s="23" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B9" s="27" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G9" s="5">
         <v>2</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>9</v>
@@ -3625,27 +3621,27 @@
         <v>6</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E10" s="21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G10" s="5">
         <v>1</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>9</v>
@@ -3654,27 +3650,27 @@
         <v>6</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>248</v>
+        <v>106</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>249</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G11" s="5">
         <v>1</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>9</v>
@@ -3683,27 +3679,27 @@
         <v>6</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G12" s="5">
         <v>1</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>9</v>
@@ -3712,27 +3708,27 @@
         <v>6</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G13" s="5">
         <v>1</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>9</v>
@@ -3741,27 +3737,27 @@
         <v>6</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G14" s="5">
         <v>2</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>9</v>
@@ -3770,27 +3766,27 @@
         <v>6</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G15" s="5">
         <v>1</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>9</v>
@@ -3799,27 +3795,27 @@
         <v>10</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G16" s="5">
         <v>1</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>9</v>
@@ -3828,27 +3824,27 @@
         <v>10</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G17" s="5">
         <v>1</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>9</v>
@@ -3857,27 +3853,27 @@
         <v>10</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G18" s="5">
         <v>1</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>9</v>
@@ -3886,27 +3882,27 @@
         <v>10</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G19" s="5">
         <v>1</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>9</v>
@@ -3915,27 +3911,27 @@
         <v>10</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G20" s="5">
         <v>2</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>9</v>
@@ -3944,27 +3940,27 @@
         <v>10</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G21" s="5">
         <v>1</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="42" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>9</v>
@@ -3973,27 +3969,27 @@
         <v>11</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E22" s="21" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G22" s="5">
         <v>3</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>9</v>
@@ -4002,27 +3998,27 @@
         <v>12</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E23" s="21" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F23" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G23" s="5">
         <v>3</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>9</v>
@@ -4031,27 +4027,27 @@
         <v>13</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>261</v>
+        <v>133</v>
+      </c>
+      <c r="E24" s="21" t="s">
+        <v>262</v>
       </c>
       <c r="F24" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G24" s="5">
         <v>2</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>9</v>
@@ -4060,27 +4056,27 @@
         <v>10</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="F25" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G25" s="5">
         <v>1</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>18</v>
@@ -4089,27 +4085,27 @@
         <v>15</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G26" s="5">
         <v>2</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>18</v>
@@ -4118,27 +4114,27 @@
         <v>15</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F27" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G27" s="5">
         <v>2</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>18</v>
@@ -4147,27 +4143,27 @@
         <v>15</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F28" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G28" s="5">
         <v>2</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>18</v>
@@ -4176,27 +4172,27 @@
         <v>15</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F29" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G29" s="5">
         <v>2</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>18</v>
@@ -4205,27 +4201,27 @@
         <v>19</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F30" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G30" s="5">
         <v>3</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>18</v>
@@ -4234,27 +4230,27 @@
         <v>19</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E31" s="21" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F31" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G31" s="5">
         <v>2</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>18</v>
@@ -4263,27 +4259,27 @@
         <v>22</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E32" s="21" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F32" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G32" s="5">
         <v>2</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>18</v>
@@ -4292,27 +4288,27 @@
         <v>24</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F33" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G33" s="5">
         <v>3</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>18</v>
@@ -4321,27 +4317,27 @@
         <v>19</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F34" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G34" s="5">
         <v>2</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>18</v>
@@ -4350,27 +4346,27 @@
         <v>25</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F35" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G35" s="5">
         <v>2</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>18</v>
@@ -4379,27 +4375,27 @@
         <v>28</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F36" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G36" s="5">
         <v>1</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>18</v>
@@ -4408,27 +4404,27 @@
         <v>28</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F37" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G37" s="5">
         <v>2</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>18</v>
@@ -4437,27 +4433,27 @@
         <v>31</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F38" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G38" s="5">
         <v>3</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>18</v>
@@ -4466,776 +4462,776 @@
         <v>13</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F39" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G39" s="5">
         <v>1</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="E40" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B40" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>175</v>
-      </c>
       <c r="F40" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G40" s="5">
         <v>2</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B41" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="F41" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G41" s="5">
         <v>2</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B42" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C42" s="5" t="s">
-        <v>38</v>
-      </c>
       <c r="D42" s="21" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F42" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G42" s="5">
         <v>2</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D43" s="21" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F43" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G43" s="5">
         <v>2</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B44" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>185</v>
-      </c>
       <c r="F44" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G44" s="5">
         <v>2</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E45" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B45" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>188</v>
-      </c>
       <c r="F45" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G45" s="5">
         <v>3</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="E46" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B46" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>191</v>
-      </c>
       <c r="F46" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G46" s="5">
         <v>2</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D47" s="21" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F47" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G47" s="5">
         <v>2</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E48" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B48" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>196</v>
-      </c>
       <c r="F48" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G48" s="5">
         <v>3</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B49" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="F49" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G49" s="5">
         <v>1</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B50" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>202</v>
-      </c>
       <c r="F50" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G50" s="5">
         <v>3</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G51" s="5">
         <v>1</v>
       </c>
       <c r="H51" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F52" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G52" s="5">
         <v>2</v>
       </c>
       <c r="H52" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E53" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="B53" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>209</v>
-      </c>
       <c r="F53" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G53" s="5">
         <v>2</v>
       </c>
       <c r="H53" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F54" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G54" s="5">
         <v>1</v>
       </c>
       <c r="H54" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="E55" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="B55" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>215</v>
-      </c>
       <c r="F55" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G55" s="5">
         <v>2</v>
       </c>
       <c r="H55" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="B56" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>218</v>
-      </c>
       <c r="F56" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G56" s="5">
         <v>2</v>
       </c>
       <c r="H56" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E57" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="B57" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>221</v>
-      </c>
       <c r="F57" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G57" s="5">
         <v>1</v>
       </c>
       <c r="H57" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B58" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="F58" s="24" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="G58" s="5">
         <v>1</v>
       </c>
       <c r="H58" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="E59" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B59" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E59" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="F59" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G59" s="5">
         <v>2</v>
       </c>
       <c r="H59" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E60" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="B60" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>230</v>
-      </c>
       <c r="F60" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G60" s="5">
         <v>1</v>
       </c>
       <c r="H60" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>378</v>
+        <v>230</v>
+      </c>
+      <c r="E61" s="21" t="s">
+        <v>273</v>
       </c>
       <c r="F61" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G61" s="5">
         <v>1</v>
       </c>
       <c r="H61" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>379</v>
+        <v>233</v>
+      </c>
+      <c r="E62" s="21" t="s">
+        <v>274</v>
       </c>
       <c r="F62" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G62" s="5">
         <v>2</v>
       </c>
       <c r="H62" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I62" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="E63" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B63" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>380</v>
-      </c>
       <c r="F63" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G63" s="5">
         <v>3</v>
       </c>
       <c r="H63" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="28" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D64" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B64" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="E64" s="3" t="s">
-        <v>381</v>
+      <c r="E64" s="21" t="s">
+        <v>275</v>
       </c>
       <c r="F64" s="24" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G64" s="5">
         <v>2</v>
       </c>
       <c r="H64" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D65" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="B65" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D65" s="3" t="s">
+      <c r="E65" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="E65" s="3" t="s">
-        <v>382</v>
-      </c>
       <c r="F65" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G65" s="5">
         <v>1</v>
       </c>
       <c r="H65" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I65" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="28" x14ac:dyDescent="0.2">
@@ -5243,46 +5239,46 @@
         <v>242</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>243</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>383</v>
+        <v>244</v>
       </c>
       <c r="F66" s="24" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G66" s="5">
         <v>1</v>
       </c>
       <c r="H66" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E68" s="10" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F68" s="11">
-        <f>COUNTA(A10:A66)</f>
-        <v>57</v>
+        <f>COUNTA(A4:A66)</f>
+        <v>63</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E69" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F69" s="11">
-        <f>SUM(G10:G66)</f>
-        <v>101</v>
+        <f>SUM(G4:G66)</f>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -5310,7 +5306,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="49" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="B1" s="49"/>
       <c r="C1" s="32"/>
@@ -5324,27 +5320,27 @@
         <v>5</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="C4" s="5" cm="1">
         <f t="array" ref="C4">SUMPRODUCT((Tickets!B$4:B$66=A4)*(Tickets!G$4:G$66))</f>
@@ -5368,7 +5364,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C5" s="5" cm="1">
         <f t="array" ref="C5">SUMPRODUCT((Tickets!B$4:B$66=A5)*(Tickets!G$4:G$66))</f>
@@ -5392,7 +5388,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C6" s="5" cm="1">
         <f t="array" ref="C6">SUMPRODUCT((Tickets!B$4:B$66=A6)*(Tickets!G$4:G$66))</f>
@@ -5413,10 +5409,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C7" s="5" cm="1">
         <f t="array" ref="C7">SUMPRODUCT((Tickets!B$4:B$66=A7)*(Tickets!G$4:G$66))</f>
@@ -5437,10 +5433,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C8" s="5" cm="1">
         <f t="array" ref="C8">SUMPRODUCT((Tickets!B$4:B$66=A8)*(Tickets!G$4:G$66))</f>
@@ -5461,7 +5457,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2">
@@ -5483,7 +5479,7 @@
     </row>
     <row r="11" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="50" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B11" s="51"/>
       <c r="C11" s="32"/>
@@ -5494,10 +5490,10 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>9</v>
@@ -5506,18 +5502,18 @@
         <v>18</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B13" s="5" cm="1">
         <f t="array" ref="B13">SUMPRODUCT((Tickets!$F$4:$F$66=$A13)*(Tickets!$B$4:$B$66=B$12)*(Tickets!$G$4:$G$66))</f>
@@ -5546,7 +5542,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B14" s="5" cm="1">
         <f t="array" ref="B14">SUMPRODUCT((Tickets!$F$4:$F$66=$A14)*(Tickets!$B$4:$B$66=B$12)*(Tickets!$G$4:$G$66))</f>
@@ -5575,7 +5571,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="B15" s="5" cm="1">
         <f t="array" ref="B15">SUMPRODUCT((Tickets!$F$4:$F$66=$A15)*(Tickets!$B$4:$B$66=B$12)*(Tickets!$G$4:$G$66))</f>
@@ -5604,7 +5600,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B16" s="2">
         <f t="shared" ref="B16:G16" si="2">SUM(B13:B15)</f>

</xml_diff>